<commit_message>
rerun all reduced tillage factors for SOC and soil erosion at raster level. SOC reduced tillage also averages
</commit_message>
<xml_diff>
--- a/data/crops/lu_c_factor_inventory.xlsx
+++ b/data/crops/lu_c_factor_inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldwildlifefund-my.sharepoint.com/personal/cristobal_loyola_wwfus_org/Documents/Documents/203. Python projects/SBTN_Test/data/crops/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="209" documentId="8_{AA2EB21E-9C36-413E-A92A-3D12D76AAA96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{222691F9-9D3B-4F39-9C0E-A780B282291D}"/>
+  <xr:revisionPtr revIDLastSave="211" documentId="8_{AA2EB21E-9C36-413E-A92A-3D12D76AAA96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{563EFAE6-9E1B-4F5C-A7AC-F25B3E3E032A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6F9D02B0-B27B-4DAB-8C90-F4F799F4886A}"/>
   </bookViews>
@@ -1830,7 +1830,18 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B91ACB39-A6C6-4049-8B69-94BB57FE429E}" name="foreground_occupation_file_index" displayName="foreground_occupation_file_index" ref="A1:M81" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:M81" xr:uid="{B91ACB39-A6C6-4049-8B69-94BB57FE429E}"/>
+  <autoFilter ref="A1:M81" xr:uid="{B91ACB39-A6C6-4049-8B69-94BB57FE429E}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="Rainfed"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="6">
+      <filters>
+        <filter val="annual_crop"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{705AD7F1-810F-4078-AF9D-E2A5540C1883}" uniqueName="1" name="file_name" queryTableFieldId="1" dataDxfId="10"/>
     <tableColumn id="2" xr3:uid="{058DBECE-D8A6-44ED-99FF-D660796ED3BB}" uniqueName="2" name="land_use" queryTableFieldId="2" dataDxfId="9"/>
@@ -2225,7 +2236,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>324</v>
       </c>
@@ -2264,7 +2275,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>325</v>
       </c>
@@ -2303,7 +2314,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>326</v>
       </c>
@@ -2342,7 +2353,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>327</v>
       </c>
@@ -2381,7 +2392,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>328</v>
       </c>
@@ -2420,7 +2431,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>329</v>
       </c>
@@ -2459,7 +2470,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>330</v>
       </c>
@@ -2498,7 +2509,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>331</v>
       </c>
@@ -2537,7 +2548,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>332</v>
       </c>
@@ -2576,7 +2587,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>333</v>
       </c>
@@ -2619,7 +2630,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>334</v>
       </c>
@@ -2662,7 +2673,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>335</v>
       </c>
@@ -2706,7 +2717,7 @@
         <v>0.17600000000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>336</v>
       </c>
@@ -2749,7 +2760,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>337</v>
       </c>
@@ -2792,7 +2803,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>338</v>
       </c>
@@ -2835,7 +2846,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>339</v>
       </c>
@@ -2878,7 +2889,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>340</v>
       </c>
@@ -2921,7 +2932,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>341</v>
       </c>
@@ -2964,7 +2975,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>342</v>
       </c>
@@ -3007,7 +3018,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>343</v>
       </c>
@@ -3050,7 +3061,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>344</v>
       </c>
@@ -3093,7 +3104,7 @@
         <v>0.32</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>345</v>
       </c>
@@ -3137,7 +3148,7 @@
         <v>0.33440000000000003</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>346</v>
       </c>
@@ -3180,7 +3191,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>347</v>
       </c>
@@ -3223,7 +3234,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>348</v>
       </c>
@@ -3266,7 +3277,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>349</v>
       </c>
@@ -3309,7 +3320,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>350</v>
       </c>
@@ -3352,7 +3363,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>351</v>
       </c>
@@ -3395,7 +3406,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>352</v>
       </c>
@@ -3439,7 +3450,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>353</v>
       </c>
@@ -3482,7 +3493,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>354</v>
       </c>
@@ -3525,7 +3536,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>355</v>
       </c>
@@ -3569,7 +3580,7 @@
         <v>8.8000000000000009E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>356</v>
       </c>
@@ -3612,7 +3623,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>357</v>
       </c>
@@ -3655,7 +3666,7 @@
         <v>0.32</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>358</v>
       </c>
@@ -3698,7 +3709,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>359</v>
       </c>
@@ -3741,7 +3752,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>360</v>
       </c>
@@ -3784,7 +3795,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>361</v>
       </c>
@@ -3827,7 +3838,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>362</v>
       </c>
@@ -3870,7 +3881,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>363</v>
       </c>
@@ -3913,7 +3924,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>364</v>
       </c>
@@ -3957,7 +3968,7 @@
         <v>0.17600000000000002</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>365</v>
       </c>
@@ -4000,7 +4011,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>366</v>
       </c>
@@ -4039,7 +4050,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>367</v>
       </c>
@@ -4078,7 +4089,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>368</v>
       </c>
@@ -4117,7 +4128,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>369</v>
       </c>
@@ -4156,7 +4167,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>370</v>
       </c>
@@ -4195,7 +4206,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>371</v>
       </c>
@@ -4234,7 +4245,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>372</v>
       </c>
@@ -4273,7 +4284,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>373</v>
       </c>
@@ -4319,7 +4330,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>374</v>
       </c>
@@ -4458,7 +4469,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>377</v>
       </c>
@@ -4504,7 +4515,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>378</v>
       </c>
@@ -4550,7 +4561,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>379</v>
       </c>
@@ -4642,7 +4653,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>381</v>
       </c>
@@ -4827,7 +4838,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>385</v>
       </c>
@@ -4873,7 +4884,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>386</v>
       </c>
@@ -4919,7 +4930,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>387</v>
       </c>
@@ -5335,7 +5346,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>396</v>
       </c>
@@ -5658,7 +5669,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>403</v>
       </c>

</xml_diff>

<commit_message>
rename SOC files. Found out C-factors are not being correctly incorporated
</commit_message>
<xml_diff>
--- a/data/crops/lu_c_factor_inventory.xlsx
+++ b/data/crops/lu_c_factor_inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldwildlifefund-my.sharepoint.com/personal/cristobal_loyola_wwfus_org/Documents/Documents/203. Python projects/SBTN_Test/data/crops/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="211" documentId="8_{AA2EB21E-9C36-413E-A92A-3D12D76AAA96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{563EFAE6-9E1B-4F5C-A7AC-F25B3E3E032A}"/>
+  <xr:revisionPtr revIDLastSave="214" documentId="8_{AA2EB21E-9C36-413E-A92A-3D12D76AAA96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC116040-C229-451C-B55F-B06B2F63D667}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6F9D02B0-B27B-4DAB-8C90-F4F799F4886A}"/>
   </bookViews>
@@ -1830,18 +1830,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B91ACB39-A6C6-4049-8B69-94BB57FE429E}" name="foreground_occupation_file_index" displayName="foreground_occupation_file_index" ref="A1:M81" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:M81" xr:uid="{B91ACB39-A6C6-4049-8B69-94BB57FE429E}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="Rainfed"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="6">
-      <filters>
-        <filter val="annual_crop"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:M81" xr:uid="{B91ACB39-A6C6-4049-8B69-94BB57FE429E}"/>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{705AD7F1-810F-4078-AF9D-E2A5540C1883}" uniqueName="1" name="file_name" queryTableFieldId="1" dataDxfId="10"/>
     <tableColumn id="2" xr3:uid="{058DBECE-D8A6-44ED-99FF-D660796ED3BB}" uniqueName="2" name="land_use" queryTableFieldId="2" dataDxfId="9"/>
@@ -2236,7 +2225,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="2" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>324</v>
       </c>
@@ -2275,7 +2264,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>325</v>
       </c>
@@ -2314,7 +2303,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>326</v>
       </c>
@@ -2353,7 +2342,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>327</v>
       </c>
@@ -2392,7 +2381,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>328</v>
       </c>
@@ -2431,7 +2420,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>329</v>
       </c>
@@ -2470,7 +2459,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>330</v>
       </c>
@@ -2509,7 +2498,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>331</v>
       </c>
@@ -2548,7 +2537,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>332</v>
       </c>
@@ -2587,7 +2576,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="11" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>333</v>
       </c>
@@ -2630,7 +2619,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="12" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>334</v>
       </c>
@@ -2673,7 +2662,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="13" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>335</v>
       </c>
@@ -2717,7 +2706,7 @@
         <v>0.17600000000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>336</v>
       </c>
@@ -2760,7 +2749,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="15" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>337</v>
       </c>
@@ -2803,7 +2792,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="16" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>338</v>
       </c>
@@ -2846,7 +2835,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>339</v>
       </c>
@@ -2889,7 +2878,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>340</v>
       </c>
@@ -2932,7 +2921,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="19" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>341</v>
       </c>
@@ -2975,7 +2964,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>342</v>
       </c>
@@ -3018,7 +3007,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>343</v>
       </c>
@@ -3061,7 +3050,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>344</v>
       </c>
@@ -3104,7 +3093,7 @@
         <v>0.32</v>
       </c>
     </row>
-    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>345</v>
       </c>
@@ -3148,7 +3137,7 @@
         <v>0.33440000000000003</v>
       </c>
     </row>
-    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>346</v>
       </c>
@@ -3191,7 +3180,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>347</v>
       </c>
@@ -3234,7 +3223,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>348</v>
       </c>
@@ -3277,7 +3266,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>349</v>
       </c>
@@ -3320,7 +3309,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>350</v>
       </c>
@@ -3363,7 +3352,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>351</v>
       </c>
@@ -3406,7 +3395,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="30" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>352</v>
       </c>
@@ -3450,7 +3439,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="31" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>353</v>
       </c>
@@ -3493,7 +3482,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>354</v>
       </c>
@@ -3536,7 +3525,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="33" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>355</v>
       </c>
@@ -3580,7 +3569,7 @@
         <v>8.8000000000000009E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>356</v>
       </c>
@@ -3623,7 +3612,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="35" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>357</v>
       </c>
@@ -3666,7 +3655,7 @@
         <v>0.32</v>
       </c>
     </row>
-    <row r="36" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>358</v>
       </c>
@@ -3709,7 +3698,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="37" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>359</v>
       </c>
@@ -3752,7 +3741,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="38" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>360</v>
       </c>
@@ -3795,7 +3784,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="39" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>361</v>
       </c>
@@ -3838,7 +3827,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="40" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>362</v>
       </c>
@@ -3881,7 +3870,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="41" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>363</v>
       </c>
@@ -3924,7 +3913,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="42" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>364</v>
       </c>
@@ -3968,7 +3957,7 @@
         <v>0.17600000000000002</v>
       </c>
     </row>
-    <row r="43" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>365</v>
       </c>
@@ -4011,7 +4000,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="44" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>366</v>
       </c>
@@ -4050,7 +4039,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="45" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>367</v>
       </c>
@@ -4089,7 +4078,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="46" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>368</v>
       </c>
@@ -4128,7 +4117,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="47" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>369</v>
       </c>
@@ -4167,7 +4156,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="48" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>370</v>
       </c>
@@ -4206,7 +4195,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="49" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>371</v>
       </c>
@@ -4245,7 +4234,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="50" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>372</v>
       </c>
@@ -4284,7 +4273,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="51" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>373</v>
       </c>
@@ -4330,7 +4319,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="52" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>374</v>
       </c>
@@ -4469,7 +4458,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="55" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>377</v>
       </c>
@@ -4515,7 +4504,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="56" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>378</v>
       </c>
@@ -4561,7 +4550,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="57" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>379</v>
       </c>
@@ -4653,7 +4642,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="59" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>381</v>
       </c>
@@ -4838,7 +4827,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="63" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>385</v>
       </c>
@@ -4884,7 +4873,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="64" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>386</v>
       </c>
@@ -4930,7 +4919,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="65" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>387</v>
       </c>
@@ -5346,7 +5335,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="74" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>396</v>
       </c>
@@ -5669,7 +5658,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="81" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>403</v>
       </c>

</xml_diff>

<commit_message>
updated lu in lu_c_factor files
</commit_message>
<xml_diff>
--- a/data/crops/lu_c_factor_inventory.xlsx
+++ b/data/crops/lu_c_factor_inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldwildlifefund-my.sharepoint.com/personal/cristobal_loyola_wwfus_org/Documents/Documents/203. Python projects/SBTN_Test/data/crops/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="214" documentId="8_{AA2EB21E-9C36-413E-A92A-3D12D76AAA96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC116040-C229-451C-B55F-B06B2F63D667}"/>
+  <xr:revisionPtr revIDLastSave="236" documentId="8_{AA2EB21E-9C36-413E-A92A-3D12D76AAA96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5721246-14B3-4A99-B1EB-AC12F47ADEC9}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6F9D02B0-B27B-4DAB-8C90-F4F799F4886A}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="863" uniqueCount="487">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="863" uniqueCount="486">
   <si>
     <t>file_name</t>
   </si>
@@ -1435,9 +1435,6 @@
   </si>
   <si>
     <t>C:\Users\loyola\OneDrive - World Wildlife Fund, Inc\Documents\203. Python projects\SBTN_Test\data\land_use\FAO_GAEZ/lu_gaez_Tomato_irr.tif</t>
-  </si>
-  <si>
-    <t>C:\Users\loyola\OneDrive - World Wildlife Fund, Inc\Documents\203. Python projects\SBTN_Test\data\land_use\FAO_GAEZ/lu_gaez_Wheat_irr_ron.tif</t>
   </si>
   <si>
     <t>C:\Users\loyola\OneDrive - World Wildlife Fund, Inc\Documents\203. Python projects\SBTN_Test\data\land_use\FAO_GAEZ/lu_gaez_Wheat_irr_roff.tif</t>
@@ -2627,7 +2624,7 @@
         <v>13</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="D12" t="s">
         <v>93</v>
@@ -2843,7 +2840,7 @@
         <v>18</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="D17" t="s">
         <v>96</v>
@@ -2886,7 +2883,7 @@
         <v>19</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="D18" t="s">
         <v>97</v>
@@ -2929,7 +2926,7 @@
         <v>20</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D19" t="s">
         <v>98</v>
@@ -3058,7 +3055,7 @@
         <v>23</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="D22" t="s">
         <v>101</v>
@@ -3188,7 +3185,7 @@
         <v>26</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="D25" t="s">
         <v>102</v>
@@ -3231,7 +3228,7 @@
         <v>27</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D26" t="s">
         <v>103</v>
@@ -3317,7 +3314,7 @@
         <v>29</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="D28" t="s">
         <v>105</v>
@@ -3447,7 +3444,7 @@
         <v>32</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="D31" t="s">
         <v>217</v>
@@ -3706,7 +3703,7 @@
         <v>38</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="D37" t="s">
         <v>110</v>
@@ -3965,7 +3962,7 @@
         <v>44</v>
       </c>
       <c r="C43" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="D43" t="s">
         <v>84</v>
@@ -4327,7 +4324,7 @@
         <v>53</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="D52" t="s">
         <v>93</v>
@@ -4373,7 +4370,7 @@
         <v>54</v>
       </c>
       <c r="C53" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="D53" t="s">
         <v>127</v>
@@ -4420,7 +4417,7 @@
         <v>55</v>
       </c>
       <c r="C54" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="D54" t="s">
         <v>127</v>
@@ -4466,7 +4463,7 @@
         <v>56</v>
       </c>
       <c r="C55" s="11" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="D55" t="s">
         <v>96</v>
@@ -4512,7 +4509,7 @@
         <v>57</v>
       </c>
       <c r="C56" s="11" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="D56" t="s">
         <v>97</v>
@@ -4558,7 +4555,7 @@
         <v>58</v>
       </c>
       <c r="C57" s="11" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="D57" t="s">
         <v>98</v>
@@ -4604,7 +4601,7 @@
         <v>59</v>
       </c>
       <c r="C58" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="D58" t="s">
         <v>99</v>
@@ -4696,7 +4693,7 @@
         <v>61</v>
       </c>
       <c r="C60" s="11" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="D60" t="s">
         <v>101</v>
@@ -4742,7 +4739,7 @@
         <v>62</v>
       </c>
       <c r="C61" s="11" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="D61" t="s">
         <v>138</v>
@@ -4789,7 +4786,7 @@
         <v>63</v>
       </c>
       <c r="C62" s="11" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="D62" t="s">
         <v>138</v>
@@ -4835,7 +4832,7 @@
         <v>64</v>
       </c>
       <c r="C63" s="11" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="D63" t="s">
         <v>102</v>
@@ -4881,7 +4878,7 @@
         <v>65</v>
       </c>
       <c r="C64" s="11" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="D64" t="s">
         <v>103</v>
@@ -4927,7 +4924,7 @@
         <v>66</v>
       </c>
       <c r="C65" s="11" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="D65" t="s">
         <v>105</v>
@@ -4973,7 +4970,7 @@
         <v>67</v>
       </c>
       <c r="C66" s="11" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="D66" t="s">
         <v>106</v>
@@ -5019,7 +5016,7 @@
         <v>68</v>
       </c>
       <c r="C67" s="11" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="D67" t="s">
         <v>217</v>
@@ -5066,7 +5063,7 @@
         <v>69</v>
       </c>
       <c r="C68" s="11" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="D68" t="s">
         <v>217</v>
@@ -5158,7 +5155,7 @@
         <v>71</v>
       </c>
       <c r="C70" s="11" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="D70" t="s">
         <v>128</v>
@@ -5205,7 +5202,7 @@
         <v>72</v>
       </c>
       <c r="C71" s="11" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="D71" t="s">
         <v>128</v>
@@ -5251,7 +5248,7 @@
         <v>73</v>
       </c>
       <c r="C72" s="11" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D72" t="s">
         <v>108</v>
@@ -5297,7 +5294,7 @@
         <v>74</v>
       </c>
       <c r="C73" s="11" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="D73" t="s">
         <v>109</v>
@@ -5343,7 +5340,7 @@
         <v>75</v>
       </c>
       <c r="C74" s="11" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="D74" t="s">
         <v>110</v>
@@ -5389,7 +5386,7 @@
         <v>76</v>
       </c>
       <c r="C75" s="11" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="D75" t="s">
         <v>111</v>
@@ -5435,7 +5432,7 @@
         <v>77</v>
       </c>
       <c r="C76" s="11" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="D76" t="s">
         <v>112</v>
@@ -5481,7 +5478,7 @@
         <v>78</v>
       </c>
       <c r="C77" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="D77" t="s">
         <v>113</v>
@@ -5527,7 +5524,7 @@
         <v>79</v>
       </c>
       <c r="C78" s="11" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="D78" t="s">
         <v>114</v>
@@ -5573,7 +5570,7 @@
         <v>80</v>
       </c>
       <c r="C79" s="11" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="D79" t="s">
         <v>84</v>
@@ -5620,7 +5617,7 @@
         <v>81</v>
       </c>
       <c r="C80" s="11" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="D80" t="s">
         <v>84</v>
@@ -5698,8 +5695,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>